<commit_message>
Ajuste en codigo diferencias para que aparezca la factura en los casos donde el importe es mayor a 20k en Colombia, y importe de facture con decimales, y otros
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_D1.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_D1.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>14/10/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2109,16 +2109,16 @@
     <row r="78">
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1259010</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
@@ -2127,178 +2127,13 @@
       </c>
       <c r="G78" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H78" s="6" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="I78" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="C79" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D79" s="10" t="inlineStr">
-        <is>
-          <t>PMP1259423</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F79" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G79" s="10" t="inlineStr">
-        <is>
-          <t>384</t>
-        </is>
-      </c>
-      <c r="H79" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I79" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>PMP1259426</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F80" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G80" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I80" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="C81" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D81" s="10" t="inlineStr">
-        <is>
-          <t>PMP1260597</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F81" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G81" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H81" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I81" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D82" s="10" t="inlineStr">
-        <is>
-          <t>PMP1260962</t>
-        </is>
-      </c>
-      <c r="E82" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F82" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G82" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H82" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I82" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="C83" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D83" s="10" t="inlineStr">
-        <is>
-          <t>PMP1261062</t>
-        </is>
-      </c>
-      <c r="E83" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F83" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G83" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H83" s="6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I83" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>

</xml_diff>

<commit_message>
Ajuste campo Descuentos en D1
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_D1.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_D1.xlsx
@@ -651,11 +651,7 @@
       <c r="E19" s="6" t="n">
         <v>25655163</v>
       </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F19" s="10" t="inlineStr"/>
       <c r="G19" s="10" t="inlineStr"/>
       <c r="H19" s="6" t="n">
         <v>25655163</v>
@@ -676,11 +672,7 @@
       <c r="E20" s="6" t="n">
         <v>2170846</v>
       </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F20" s="10" t="inlineStr"/>
       <c r="G20" s="10" t="inlineStr"/>
       <c r="H20" s="6" t="n">
         <v>2170846</v>
@@ -701,11 +693,7 @@
       <c r="E21" s="6" t="n">
         <v>4096575</v>
       </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F21" s="10" t="inlineStr"/>
       <c r="G21" s="10" t="inlineStr"/>
       <c r="H21" s="6" t="n">
         <v>4096575</v>
@@ -726,11 +714,7 @@
       <c r="E22" s="6" t="n">
         <v>37979893</v>
       </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F22" s="10" t="inlineStr"/>
       <c r="G22" s="10" t="inlineStr"/>
       <c r="H22" s="6" t="n">
         <v>37979893</v>
@@ -751,11 +735,7 @@
       <c r="E23" s="6" t="n">
         <v>5427114</v>
       </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F23" s="10" t="inlineStr"/>
       <c r="G23" s="10" t="inlineStr"/>
       <c r="H23" s="6" t="n">
         <v>5427114</v>
@@ -776,11 +756,7 @@
       <c r="E24" s="6" t="n">
         <v>38950128</v>
       </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F24" s="10" t="inlineStr"/>
       <c r="G24" s="10" t="inlineStr"/>
       <c r="H24" s="6" t="n">
         <v>38950128</v>
@@ -801,11 +777,7 @@
       <c r="E25" s="6" t="n">
         <v>33682950</v>
       </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F25" s="10" t="inlineStr"/>
       <c r="G25" s="10" t="inlineStr"/>
       <c r="H25" s="6" t="n">
         <v>33682950</v>
@@ -826,11 +798,7 @@
       <c r="E26" s="6" t="n">
         <v>6303830</v>
       </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F26" s="10" t="inlineStr"/>
       <c r="G26" s="10" t="inlineStr"/>
       <c r="H26" s="6" t="n">
         <v>6303830</v>
@@ -851,11 +819,7 @@
       <c r="E27" s="6" t="n">
         <v>78357242</v>
       </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F27" s="10" t="inlineStr"/>
       <c r="G27" s="10" t="inlineStr"/>
       <c r="H27" s="6" t="n">
         <v>78357242</v>
@@ -876,11 +840,7 @@
       <c r="E28" s="6" t="n">
         <v>5427114</v>
       </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F28" s="10" t="inlineStr"/>
       <c r="G28" s="10" t="inlineStr"/>
       <c r="H28" s="6" t="n">
         <v>5427114</v>
@@ -901,11 +861,7 @@
       <c r="E29" s="6" t="n">
         <v>41776426</v>
       </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F29" s="10" t="inlineStr"/>
       <c r="G29" s="10" t="inlineStr"/>
       <c r="H29" s="6" t="n">
         <v>41776426</v>
@@ -926,11 +882,7 @@
       <c r="E30" s="6" t="n">
         <v>5462100</v>
       </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F30" s="10" t="inlineStr"/>
       <c r="G30" s="10" t="inlineStr"/>
       <c r="H30" s="6" t="n">
         <v>5462100</v>
@@ -951,11 +903,7 @@
       <c r="E31" s="6" t="n">
         <v>8683382</v>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F31" s="10" t="inlineStr"/>
       <c r="G31" s="10" t="inlineStr"/>
       <c r="H31" s="6" t="n">
         <v>8683382</v>
@@ -976,11 +924,7 @@
       <c r="E32" s="6" t="n">
         <v>23220422</v>
       </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F32" s="10" t="inlineStr"/>
       <c r="G32" s="10" t="inlineStr"/>
       <c r="H32" s="6" t="n">
         <v>23220422</v>
@@ -1001,11 +945,7 @@
       <c r="E33" s="6" t="n">
         <v>6827625</v>
       </c>
-      <c r="F33" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F33" s="10" t="inlineStr"/>
       <c r="G33" s="10" t="inlineStr"/>
       <c r="H33" s="6" t="n">
         <v>6827625</v>
@@ -1026,11 +966,7 @@
       <c r="E34" s="6" t="n">
         <v>14110425</v>
       </c>
-      <c r="F34" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F34" s="10" t="inlineStr"/>
       <c r="G34" s="10" t="inlineStr"/>
       <c r="H34" s="6" t="n">
         <v>14110425</v>
@@ -1051,11 +987,7 @@
       <c r="E35" s="6" t="n">
         <v>8683382</v>
       </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F35" s="10" t="inlineStr"/>
       <c r="G35" s="10" t="inlineStr"/>
       <c r="H35" s="6" t="n">
         <v>8683382</v>
@@ -1076,11 +1008,7 @@
       <c r="E36" s="6" t="n">
         <v>12975535</v>
       </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F36" s="10" t="inlineStr"/>
       <c r="G36" s="10" t="inlineStr"/>
       <c r="H36" s="6" t="n">
         <v>12975535</v>
@@ -1101,11 +1029,7 @@
       <c r="E37" s="6" t="n">
         <v>17258914</v>
       </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F37" s="10" t="inlineStr"/>
       <c r="G37" s="10" t="inlineStr"/>
       <c r="H37" s="6" t="n">
         <v>17258914</v>
@@ -1126,11 +1050,7 @@
       <c r="E38" s="6" t="n">
         <v>52433082</v>
       </c>
-      <c r="F38" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F38" s="10" t="inlineStr"/>
       <c r="G38" s="10" t="inlineStr"/>
       <c r="H38" s="6" t="n">
         <v>52433082</v>
@@ -1151,11 +1071,7 @@
       <c r="E39" s="6" t="n">
         <v>39584477</v>
       </c>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F39" s="10" t="inlineStr"/>
       <c r="G39" s="10" t="inlineStr"/>
       <c r="H39" s="6" t="n">
         <v>39584477</v>
@@ -1176,11 +1092,7 @@
       <c r="E40" s="6" t="n">
         <v>27160433</v>
       </c>
-      <c r="F40" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F40" s="10" t="inlineStr"/>
       <c r="G40" s="10" t="inlineStr"/>
       <c r="H40" s="6" t="n">
         <v>27160433</v>
@@ -1201,11 +1113,7 @@
       <c r="E41" s="6" t="n">
         <v>1628134</v>
       </c>
-      <c r="F41" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F41" s="10" t="inlineStr"/>
       <c r="G41" s="10" t="inlineStr"/>
       <c r="H41" s="6" t="n">
         <v>1628134</v>
@@ -1226,11 +1134,7 @@
       <c r="E42" s="6" t="n">
         <v>8193150</v>
       </c>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F42" s="10" t="inlineStr"/>
       <c r="G42" s="10" t="inlineStr"/>
       <c r="H42" s="6" t="n">
         <v>8193150</v>
@@ -1251,11 +1155,7 @@
       <c r="E43" s="6" t="n">
         <v>17250097</v>
       </c>
-      <c r="F43" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F43" s="10" t="inlineStr"/>
       <c r="G43" s="10" t="inlineStr"/>
       <c r="H43" s="6" t="n">
         <v>17250097</v>
@@ -1276,11 +1176,7 @@
       <c r="E44" s="6" t="n">
         <v>11939651</v>
       </c>
-      <c r="F44" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F44" s="10" t="inlineStr"/>
       <c r="G44" s="10" t="inlineStr"/>
       <c r="H44" s="6" t="n">
         <v>11939651</v>
@@ -1301,11 +1197,7 @@
       <c r="E45" s="6" t="n">
         <v>35958825</v>
       </c>
-      <c r="F45" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F45" s="10" t="inlineStr"/>
       <c r="G45" s="10" t="inlineStr"/>
       <c r="H45" s="6" t="n">
         <v>35958825</v>
@@ -1326,11 +1218,7 @@
       <c r="E46" s="6" t="n">
         <v>98292747</v>
       </c>
-      <c r="F46" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F46" s="10" t="inlineStr"/>
       <c r="G46" s="10" t="inlineStr"/>
       <c r="H46" s="6" t="n">
         <v>98292747</v>
@@ -1351,11 +1239,7 @@
       <c r="E47" s="6" t="n">
         <v>3256268</v>
       </c>
-      <c r="F47" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F47" s="10" t="inlineStr"/>
       <c r="G47" s="10" t="inlineStr"/>
       <c r="H47" s="6" t="n">
         <v>3256268</v>
@@ -1376,11 +1260,7 @@
       <c r="E48" s="6" t="n">
         <v>910350</v>
       </c>
-      <c r="F48" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F48" s="10" t="inlineStr"/>
       <c r="G48" s="10" t="inlineStr"/>
       <c r="H48" s="6" t="n">
         <v>910350</v>
@@ -1401,11 +1281,7 @@
       <c r="E49" s="6" t="n">
         <v>22432167</v>
       </c>
-      <c r="F49" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F49" s="10" t="inlineStr"/>
       <c r="G49" s="10" t="inlineStr"/>
       <c r="H49" s="6" t="n">
         <v>22432167</v>
@@ -1426,11 +1302,7 @@
       <c r="E50" s="6" t="n">
         <v>5427114</v>
       </c>
-      <c r="F50" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F50" s="10" t="inlineStr"/>
       <c r="G50" s="10" t="inlineStr"/>
       <c r="H50" s="6" t="n">
         <v>5427114</v>
@@ -1451,11 +1323,7 @@
       <c r="E51" s="6" t="n">
         <v>33181151</v>
       </c>
-      <c r="F51" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F51" s="10" t="inlineStr"/>
       <c r="G51" s="10" t="inlineStr"/>
       <c r="H51" s="6" t="n">
         <v>33181151</v>
@@ -1476,11 +1344,7 @@
       <c r="E52" s="6" t="n">
         <v>19947303</v>
       </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F52" s="10" t="inlineStr"/>
       <c r="G52" s="10" t="inlineStr"/>
       <c r="H52" s="6" t="n">
         <v>19947303</v>
@@ -1501,11 +1365,7 @@
       <c r="E53" s="6" t="n">
         <v>58694897</v>
       </c>
-      <c r="F53" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F53" s="10" t="inlineStr"/>
       <c r="G53" s="10" t="inlineStr"/>
       <c r="H53" s="6" t="n">
         <v>58694897</v>
@@ -1526,11 +1386,7 @@
       <c r="E54" s="6" t="n">
         <v>52938835</v>
       </c>
-      <c r="F54" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F54" s="10" t="inlineStr"/>
       <c r="G54" s="10" t="inlineStr"/>
       <c r="H54" s="6" t="n">
         <v>52938835</v>
@@ -1551,11 +1407,7 @@
       <c r="E55" s="6" t="n">
         <v>45062325</v>
       </c>
-      <c r="F55" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F55" s="10" t="inlineStr"/>
       <c r="G55" s="10" t="inlineStr"/>
       <c r="H55" s="6" t="n">
         <v>45062325</v>
@@ -1576,11 +1428,7 @@
       <c r="E56" s="6" t="n">
         <v>11939651</v>
       </c>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F56" s="10" t="inlineStr"/>
       <c r="G56" s="10" t="inlineStr"/>
       <c r="H56" s="6" t="n">
         <v>11939651</v>
@@ -1601,11 +1449,7 @@
       <c r="E57" s="6" t="n">
         <v>47387323</v>
       </c>
-      <c r="F57" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F57" s="10" t="inlineStr"/>
       <c r="G57" s="10" t="inlineStr"/>
       <c r="H57" s="6" t="n">
         <v>47387323</v>
@@ -1626,11 +1470,7 @@
       <c r="E58" s="6" t="n">
         <v>45078536</v>
       </c>
-      <c r="F58" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F58" s="10" t="inlineStr"/>
       <c r="G58" s="10" t="inlineStr"/>
       <c r="H58" s="6" t="n">
         <v>45078536</v>
@@ -1651,11 +1491,7 @@
       <c r="E59" s="6" t="n">
         <v>23662781</v>
       </c>
-      <c r="F59" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F59" s="10" t="inlineStr"/>
       <c r="G59" s="10" t="inlineStr"/>
       <c r="H59" s="6" t="n">
         <v>23662781</v>
@@ -1676,11 +1512,7 @@
       <c r="E60" s="6" t="n">
         <v>29445126</v>
       </c>
-      <c r="F60" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F60" s="10" t="inlineStr"/>
       <c r="G60" s="10" t="inlineStr"/>
       <c r="H60" s="6" t="n">
         <v>29445126</v>
@@ -1701,11 +1533,7 @@
       <c r="E61" s="6" t="n">
         <v>32562684</v>
       </c>
-      <c r="F61" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F61" s="10" t="inlineStr"/>
       <c r="G61" s="10" t="inlineStr"/>
       <c r="H61" s="6" t="n">
         <v>32562684</v>
@@ -1726,11 +1554,7 @@
       <c r="E62" s="6" t="n">
         <v>27765675</v>
       </c>
-      <c r="F62" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F62" s="10" t="inlineStr"/>
       <c r="G62" s="10" t="inlineStr"/>
       <c r="H62" s="6" t="n">
         <v>27765675</v>
@@ -1751,11 +1575,7 @@
       <c r="E63" s="6" t="n">
         <v>41420925</v>
       </c>
-      <c r="F63" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F63" s="10" t="inlineStr"/>
       <c r="G63" s="10" t="inlineStr"/>
       <c r="H63" s="6" t="n">
         <v>41420925</v>
@@ -1776,11 +1596,7 @@
       <c r="E64" s="6" t="n">
         <v>83814032</v>
       </c>
-      <c r="F64" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F64" s="10" t="inlineStr"/>
       <c r="G64" s="10" t="inlineStr"/>
       <c r="H64" s="6" t="n">
         <v>83814032</v>
@@ -1801,11 +1617,7 @@
       <c r="E65" s="6" t="n">
         <v>34733529</v>
       </c>
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F65" s="10" t="inlineStr"/>
       <c r="G65" s="10" t="inlineStr"/>
       <c r="H65" s="6" t="n">
         <v>34733529</v>
@@ -1826,11 +1638,7 @@
       <c r="E66" s="6" t="n">
         <v>78979257</v>
       </c>
-      <c r="F66" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F66" s="10" t="inlineStr"/>
       <c r="G66" s="10" t="inlineStr"/>
       <c r="H66" s="6" t="n">
         <v>78979257</v>
@@ -1851,11 +1659,7 @@
       <c r="E67" s="6" t="n">
         <v>22793879</v>
       </c>
-      <c r="F67" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F67" s="10" t="inlineStr"/>
       <c r="G67" s="10" t="inlineStr"/>
       <c r="H67" s="6" t="n">
         <v>22793879</v>
@@ -1876,11 +1680,7 @@
       <c r="E68" s="6" t="n">
         <v>14565600</v>
       </c>
-      <c r="F68" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F68" s="10" t="inlineStr"/>
       <c r="G68" s="10" t="inlineStr"/>
       <c r="H68" s="6" t="n">
         <v>14565600</v>
@@ -1901,11 +1701,7 @@
       <c r="E69" s="6" t="n">
         <v>63624826</v>
       </c>
-      <c r="F69" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F69" s="10" t="inlineStr"/>
       <c r="G69" s="10" t="inlineStr"/>
       <c r="H69" s="6" t="n">
         <v>63624826</v>
@@ -1926,11 +1722,7 @@
       <c r="E70" s="6" t="n">
         <v>91233227</v>
       </c>
-      <c r="F70" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F70" s="10" t="inlineStr"/>
       <c r="G70" s="10" t="inlineStr"/>
       <c r="H70" s="6" t="n">
         <v>91233227</v>
@@ -1951,11 +1743,7 @@
       <c r="E71" s="6" t="n">
         <v>79868468</v>
       </c>
-      <c r="F71" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F71" s="10" t="inlineStr"/>
       <c r="G71" s="10" t="inlineStr"/>
       <c r="H71" s="6" t="n">
         <v>79868468</v>
@@ -1976,11 +1764,7 @@
       <c r="E72" s="6" t="n">
         <v>21848400</v>
       </c>
-      <c r="F72" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F72" s="10" t="inlineStr"/>
       <c r="G72" s="10" t="inlineStr"/>
       <c r="H72" s="6" t="n">
         <v>21848400</v>
@@ -2001,11 +1785,7 @@
       <c r="E73" s="6" t="n">
         <v>29306416</v>
       </c>
-      <c r="F73" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F73" s="10" t="inlineStr"/>
       <c r="G73" s="10" t="inlineStr"/>
       <c r="H73" s="6" t="n">
         <v>29306416</v>
@@ -2026,11 +1806,7 @@
       <c r="E74" s="6" t="n">
         <v>10924200</v>
       </c>
-      <c r="F74" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F74" s="10" t="inlineStr"/>
       <c r="G74" s="10" t="inlineStr"/>
       <c r="H74" s="6" t="n">
         <v>10924200</v>
@@ -2051,11 +1827,7 @@
       <c r="E75" s="6" t="n">
         <v>20623033</v>
       </c>
-      <c r="F75" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F75" s="10" t="inlineStr"/>
       <c r="G75" s="10" t="inlineStr"/>
       <c r="H75" s="6" t="n">
         <v>20623033</v>
@@ -2076,11 +1848,7 @@
       <c r="E76" s="6" t="n">
         <v>55704423</v>
       </c>
-      <c r="F76" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F76" s="10" t="inlineStr"/>
       <c r="G76" s="10" t="inlineStr"/>
       <c r="H76" s="6" t="n">
         <v>55704423</v>
@@ -2101,11 +1869,7 @@
       <c r="E77" s="6" t="n">
         <v>73484886</v>
       </c>
-      <c r="F77" s="10" t="inlineStr">
-        <is>
-          <t>Descuento</t>
-        </is>
-      </c>
+      <c r="F77" s="10" t="inlineStr"/>
       <c r="G77" s="10" t="inlineStr"/>
       <c r="H77" s="6" t="n">
         <v>73484886</v>

</xml_diff>